<commit_message>
feat(templates): update master templates with source-accurate data and tables
- Rebuild 4 master templates from raw OFM, SAEP, and ESD QCEW data sources
- Convert data ranges to native Excel Tables (ListObject) across all templates
- Enforce locked/hidden formula cells and unlocked row 8 headers
- Add data/templates/summary.md documenting rebuild methodologies and assumptions
- Refresh Star Schema data model and processed CSVs with verified AMI fact table
</commit_message>
<xml_diff>
--- a/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
+++ b/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
@@ -33961,7 +33961,7 @@
     <col width="27" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="129" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -34062,23 +34062,23 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34113,23 +34113,23 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34161,16 +34161,16 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -34180,7 +34180,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34209,19 +34209,19 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -34231,7 +34231,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34260,16 +34260,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -34278,11 +34278,11 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34317,23 +34317,23 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>4</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34384,7 +34384,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34413,16 +34413,16 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -34435,7 +34435,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34464,29 +34464,29 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>4</v>
+        <v>211</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>211</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34515,17 +34515,17 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
         <v>2</v>
       </c>
-      <c r="I11" t="n">
-        <v>1</v>
-      </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
@@ -34533,11 +34533,11 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34572,23 +34572,23 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34620,26 +34620,26 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34668,19 +34668,19 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -34690,7 +34690,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34719,19 +34719,19 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -34741,7 +34741,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34770,29 +34770,29 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
         <v>3</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34827,23 +34827,23 @@
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34875,16 +34875,16 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -34894,7 +34894,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34923,29 +34923,29 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
         <v>3</v>
       </c>
-      <c r="H19" t="n">
-        <v>4</v>
-      </c>
-      <c r="I19" t="n">
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
         <v>3</v>
       </c>
-      <c r="J19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -34974,29 +34974,29 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>
@@ -35025,17 +35025,17 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
         <v>3</v>
       </c>
-      <c r="I21" t="n">
-        <v>2</v>
-      </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
@@ -35043,11 +35043,11 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Default Allocation (WA Commerce Exhibit 12) — Local 2025 AMI datasheets not yet due (10/20); not a jurisdiction-verified split</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(etl): map OFM ADU permits correctly and retain exact valuation cents
- Correct mapping of OFM column 16 to ADU_Units instead of Mobile_Home_Units in Fact_HousingPermits
- Set Mobile_Home_Units to 0 to align with source columns and master templates
- Retain exact 2-decimal valuation cents for UGA dev permits
- Refresh Fact_HousingPermits.csv and SCOG_Star_Schema_Data_Model.xlsx
- Add docs/validation_report.md documenting cell-by-cell verification results
</commit_message>
<xml_diff>
--- a/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
+++ b/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
@@ -7769,10 +7769,10 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
         <v>40</v>
@@ -7827,10 +7827,10 @@
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K24" t="n">
         <v>38</v>
@@ -7885,10 +7885,10 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
         <v>56</v>
@@ -7943,10 +7943,10 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
         <v>54</v>
@@ -8001,10 +8001,10 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
         <v>30</v>
@@ -8059,10 +8059,10 @@
         <v>17</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J28" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
         <v>75</v>
@@ -8117,10 +8117,10 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J29" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
         <v>102</v>
@@ -8175,10 +8175,10 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J30" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
         <v>116</v>
@@ -8291,10 +8291,10 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J32" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
         <v>69</v>
@@ -8349,10 +8349,10 @@
         <v>25</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J33" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
         <v>120</v>
@@ -8465,10 +8465,10 @@
         <v>15</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J35" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
         <v>72</v>
@@ -8523,10 +8523,10 @@
         <v>38</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J36" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
         <v>74</v>
@@ -8581,10 +8581,10 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J37" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K37" t="n">
         <v>31</v>
@@ -8639,10 +8639,10 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J38" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
         <v>30</v>
@@ -10321,10 +10321,10 @@
         <v>84</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K67" t="n">
         <v>122</v>
@@ -10495,10 +10495,10 @@
         <v>236</v>
       </c>
       <c r="I70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K70" t="n">
         <v>253</v>
@@ -10553,10 +10553,10 @@
         <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K71" t="n">
         <v>15</v>
@@ -10669,10 +10669,10 @@
         <v>202</v>
       </c>
       <c r="I73" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J73" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K73" t="n">
         <v>213</v>
@@ -10727,10 +10727,10 @@
         <v>211</v>
       </c>
       <c r="I74" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J74" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K74" t="n">
         <v>217</v>
@@ -10785,10 +10785,10 @@
         <v>42</v>
       </c>
       <c r="I75" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J75" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K75" t="n">
         <v>52</v>
@@ -16875,10 +16875,10 @@
         <v>0</v>
       </c>
       <c r="I180" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J180" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K180" t="n">
         <v>7</v>
@@ -16991,10 +16991,10 @@
         <v>0</v>
       </c>
       <c r="I182" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J182" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K182" t="n">
         <v>14</v>
@@ -17165,10 +17165,10 @@
         <v>0</v>
       </c>
       <c r="I185" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J185" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K185" t="n">
         <v>3</v>
@@ -19137,10 +19137,10 @@
         <v>0</v>
       </c>
       <c r="I219" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J219" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K219" t="n">
         <v>1</v>
@@ -20703,10 +20703,10 @@
         <v>0</v>
       </c>
       <c r="I246" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J246" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K246" t="n">
         <v>111</v>
@@ -20819,10 +20819,10 @@
         <v>16</v>
       </c>
       <c r="I248" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J248" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K248" t="n">
         <v>156</v>
@@ -20935,10 +20935,10 @@
         <v>23</v>
       </c>
       <c r="I250" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J250" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K250" t="n">
         <v>156</v>
@@ -20993,10 +20993,10 @@
         <v>0</v>
       </c>
       <c r="I251" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J251" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K251" t="n">
         <v>154</v>
@@ -21051,10 +21051,10 @@
         <v>6</v>
       </c>
       <c r="I252" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J252" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K252" t="n">
         <v>118</v>
@@ -21109,10 +21109,10 @@
         <v>34</v>
       </c>
       <c r="I253" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J253" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K253" t="n">
         <v>119</v>
@@ -21167,10 +21167,10 @@
         <v>5</v>
       </c>
       <c r="I254" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J254" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K254" t="n">
         <v>106</v>
@@ -21283,10 +21283,10 @@
         <v>121</v>
       </c>
       <c r="I256" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J256" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K256" t="n">
         <v>157</v>
@@ -21341,10 +21341,10 @@
         <v>10</v>
       </c>
       <c r="I257" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J257" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K257" t="n">
         <v>27</v>
@@ -21399,10 +21399,10 @@
         <v>50</v>
       </c>
       <c r="I258" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J258" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K258" t="n">
         <v>95</v>
@@ -21457,10 +21457,10 @@
         <v>0</v>
       </c>
       <c r="I259" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J259" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K259" t="n">
         <v>23</v>
@@ -21515,10 +21515,10 @@
         <v>0</v>
       </c>
       <c r="I260" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J260" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K260" t="n">
         <v>38</v>
@@ -23371,10 +23371,10 @@
         <v>0</v>
       </c>
       <c r="I292" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J292" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K292" t="n">
         <v>63</v>
@@ -23429,10 +23429,10 @@
         <v>100</v>
       </c>
       <c r="I293" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J293" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K293" t="n">
         <v>202</v>
@@ -23487,10 +23487,10 @@
         <v>0</v>
       </c>
       <c r="I294" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J294" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K294" t="n">
         <v>42</v>
@@ -23545,10 +23545,10 @@
         <v>87</v>
       </c>
       <c r="I295" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J295" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K295" t="n">
         <v>132</v>
@@ -23603,10 +23603,10 @@
         <v>15</v>
       </c>
       <c r="I296" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J296" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K296" t="n">
         <v>56</v>
@@ -23661,10 +23661,10 @@
         <v>0</v>
       </c>
       <c r="I297" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J297" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K297" t="n">
         <v>27</v>
@@ -23737,7 +23737,7 @@
         <v>12</v>
       </c>
       <c r="O298" t="n">
-        <v>4343012</v>
+        <v>4343012.17</v>
       </c>
       <c r="P298" t="inlineStr">
         <is>
@@ -23795,7 +23795,7 @@
         <v>0</v>
       </c>
       <c r="O299" t="n">
-        <v>32637</v>
+        <v>32637.35</v>
       </c>
       <c r="P299" t="inlineStr">
         <is>
@@ -24415,10 +24415,10 @@
         <v>0</v>
       </c>
       <c r="I310" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="J310" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="K310" t="n">
         <v>63</v>
@@ -24473,10 +24473,10 @@
         <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="J311" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="K311" t="n">
         <v>153</v>
@@ -24531,10 +24531,10 @@
         <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="J312" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K312" t="n">
         <v>131</v>
@@ -24589,10 +24589,10 @@
         <v>0</v>
       </c>
       <c r="I313" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="J313" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K313" t="n">
         <v>112</v>
@@ -24647,10 +24647,10 @@
         <v>0</v>
       </c>
       <c r="I314" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="J314" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K314" t="n">
         <v>150</v>
@@ -24705,10 +24705,10 @@
         <v>0</v>
       </c>
       <c r="I315" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J315" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K315" t="n">
         <v>85</v>

</xml_diff>

<commit_message>
feat(powerbi): deliver 2025 prototype PBIP with audited governance and visual disclaimers
</commit_message>
<xml_diff>
--- a/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
+++ b/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -428,8 +428,10 @@
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,10 +462,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>County_Name</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
@@ -491,12 +503,18 @@
       <c r="E2" t="n">
         <v>1</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="n">
+        <v>48.5126</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-122.6127</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -524,12 +542,18 @@
       <c r="E3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="n">
+        <v>48.4757</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-122.3254</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -557,12 +581,18 @@
       <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="n">
+        <v>48.5393</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-121.7471</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -590,12 +620,18 @@
       <c r="E5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" t="n">
+        <v>48.5246</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-121.9868</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -623,12 +659,18 @@
       <c r="E6" t="n">
         <v>1</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" t="n">
+        <v>48.3943</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-122.4957</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -656,12 +698,18 @@
       <c r="E7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" t="n">
+        <v>48.5251</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-122.0621</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -689,12 +737,18 @@
       <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" t="n">
+        <v>48.4212</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-122.334</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -722,12 +776,18 @@
       <c r="E9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" t="n">
+        <v>48.5039</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-122.2363</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -755,12 +815,18 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" t="n">
+        <v>48.4717</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-122.4239</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -788,12 +854,18 @@
       <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" t="n">
+        <v>48.4069</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-122.5186</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
@@ -821,12 +893,18 @@
       <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" t="n">
+        <v>48.48</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-121.8</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>Skagit</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>WA</t>
         </is>

</xml_diff>

<commit_message>
fix(powerbi): derive rural population by subtracting UGAs, update display labels and footnote
</commit_message>
<xml_diff>
--- a/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
+++ b/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
@@ -424,7 +424,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -879,7 +879,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2497,7 +2497,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4037,12 +4037,12 @@
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7348,15 +7348,15 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>52606</v>
+        <v>44096</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>OFM_April1_Official_Determination</t>
+          <t>Derived (OFM Unincorporated minus UGAs)</t>
         </is>
       </c>
     </row>
@@ -7376,24 +7376,24 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>52750</v>
+        <v>48491</v>
       </c>
       <c r="F93" t="n">
-        <v>52606</v>
+        <v>44096</v>
       </c>
       <c r="G93" t="n">
-        <v>144</v>
+        <v>4395</v>
       </c>
       <c r="H93" t="n">
-        <v>0.0027</v>
+        <v>0.0997</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>OFM_April1_Official_Determination</t>
+          <t>Derived (OFM Unincorporated minus UGAs)</t>
         </is>
       </c>
     </row>
@@ -7413,24 +7413,24 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>52970</v>
+        <v>48710</v>
       </c>
       <c r="F94" t="n">
-        <v>52750</v>
+        <v>48491</v>
       </c>
       <c r="G94" t="n">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H94" t="n">
-        <v>0.0042</v>
+        <v>0.0045</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>OFM_April1_Official_Determination</t>
+          <t>Derived (OFM Unincorporated minus UGAs)</t>
         </is>
       </c>
     </row>
@@ -7450,24 +7450,24 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>53065</v>
+        <v>48799</v>
       </c>
       <c r="F95" t="n">
-        <v>52970</v>
+        <v>48710</v>
       </c>
       <c r="G95" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="H95" t="n">
         <v>0.0018</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>OFM_April1_Official_Determination</t>
+          <t>Derived (OFM Unincorporated minus UGAs)</t>
         </is>
       </c>
     </row>
@@ -7487,24 +7487,24 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>53210</v>
+        <v>48946</v>
       </c>
       <c r="F96" t="n">
-        <v>53065</v>
+        <v>48799</v>
       </c>
       <c r="G96" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H96" t="n">
-        <v>0.0027</v>
+        <v>0.003</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>OFM_April1_Official_Determination</t>
+          <t>Derived (OFM Unincorporated minus UGAs)</t>
         </is>
       </c>
     </row>
@@ -7524,24 +7524,24 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>53380</v>
+        <v>49102</v>
       </c>
       <c r="F97" t="n">
-        <v>53210</v>
+        <v>48946</v>
       </c>
       <c r="G97" t="n">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="H97" t="n">
         <v>0.0032</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>OFM_April1_Official_Determination</t>
+          <t>Derived (OFM Unincorporated minus UGAs)</t>
         </is>
       </c>
     </row>
@@ -7561,24 +7561,24 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>53580</v>
+        <v>49299</v>
       </c>
       <c r="F98" t="n">
-        <v>53380</v>
+        <v>49102</v>
       </c>
       <c r="G98" t="n">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="H98" t="n">
-        <v>0.0037</v>
+        <v>0.004</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>OFM_April1_Official_Determination</t>
+          <t>Derived (OFM Unincorporated minus UGAs)</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7599,7 @@
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -24996,7 +24996,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E300" t="n">
@@ -25054,7 +25054,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E301" t="n">
@@ -25112,7 +25112,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E302" t="n">
@@ -25170,7 +25170,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E303" t="n">
@@ -25228,7 +25228,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E304" t="n">
@@ -25286,7 +25286,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E305" t="n">
@@ -25344,7 +25344,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E306" t="n">
@@ -25402,7 +25402,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E307" t="n">
@@ -25460,7 +25460,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E308" t="n">
@@ -25518,7 +25518,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E309" t="n">
@@ -25576,7 +25576,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E310" t="n">
@@ -25634,7 +25634,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E311" t="n">
@@ -25692,7 +25692,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E312" t="n">
@@ -25750,7 +25750,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E313" t="n">
@@ -25808,7 +25808,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E314" t="n">
@@ -25866,7 +25866,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Unincorporated Skagit County</t>
+          <t>Unincorporated Rural (outside UGAs)</t>
         </is>
       </c>
       <c r="E315" t="n">

</xml_diff>

<commit_message>
fix(etl): deduplicate SAEP 2020 UGA columns and assert county total additivity 2020-2026
</commit_message>
<xml_diff>
--- a/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
+++ b/scog-growth-report/data/processed/SCOG_Star_Schema_Data_Model.xlsx
@@ -7352,7 +7352,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>44096</v>
+        <v>48351</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
@@ -7383,13 +7383,13 @@
         <v>48491</v>
       </c>
       <c r="F93" t="n">
-        <v>44096</v>
+        <v>48351</v>
       </c>
       <c r="G93" t="n">
-        <v>4395</v>
+        <v>140</v>
       </c>
       <c r="H93" t="n">
-        <v>0.0997</v>
+        <v>0.0029</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>

</xml_diff>